<commit_message>
Update Pertanggal 30 April 2026 08:53 WIB
</commit_message>
<xml_diff>
--- a/Documentation/Documents/SQL Generator/Data Initial/Master.TblBank.xlsx
+++ b/Documentation/Documents/SQL Generator/Data Initial/Master.TblBank.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6000" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6000" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="MAIN" sheetId="5" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="114">
   <si>
     <t>Mandiri</t>
   </si>
@@ -286,9 +286,6 @@
     <t>BJTMIDJA</t>
   </si>
   <si>
-    <t xml:space="preserve"> PDKSIDJ1</t>
-  </si>
-  <si>
     <t>BRI Syariah</t>
   </si>
   <si>
@@ -311,6 +308,57 @@
   </si>
   <si>
     <t>Bank Acronym</t>
+  </si>
+  <si>
+    <t>Bank Code</t>
+  </si>
+  <si>
+    <t>MRI</t>
+  </si>
+  <si>
+    <t>MEG</t>
+  </si>
+  <si>
+    <t>PER</t>
+  </si>
+  <si>
+    <t>DAN</t>
+  </si>
+  <si>
+    <t>BUK</t>
+  </si>
+  <si>
+    <t>OCB</t>
+  </si>
+  <si>
+    <t>TPN</t>
+  </si>
+  <si>
+    <t>PAN</t>
+  </si>
+  <si>
+    <t>MAY</t>
+  </si>
+  <si>
+    <t>CMW</t>
+  </si>
+  <si>
+    <t>SCD</t>
+  </si>
+  <si>
+    <t>CIM</t>
+  </si>
+  <si>
+    <t>RIS</t>
+  </si>
+  <si>
+    <t>PDB</t>
+  </si>
+  <si>
+    <t>PDJ</t>
+  </si>
+  <si>
+    <t>PDK</t>
   </si>
 </sst>
 </file>
@@ -604,7 +652,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -661,6 +709,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -996,7 +1047,7 @@
     </row>
     <row r="2" spans="2:7" s="6" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="B2" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>41</v>
@@ -1005,10 +1056,10 @@
         <v>39</v>
       </c>
       <c r="F2" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="G2" s="12" t="s">
         <v>93</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="3" spans="2:7" s="6" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -1313,7 +1364,7 @@
         <v>37</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D20" s="17" t="s">
         <v>38</v>
@@ -1332,7 +1383,7 @@
         <v>73</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D21" s="17" t="s">
         <v>85</v>
@@ -1411,7 +1462,7 @@
         <v>78</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F25" s="15">
         <f t="shared" si="0"/>
@@ -1456,13 +1507,13 @@
     <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="D2" s="32" t="s">
         <v>96</v>
-      </c>
-      <c r="C2" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" s="32" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1790,20 +1841,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:G23"/>
+  <dimension ref="B1:J23"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="3"/>
     <col min="2" max="2" width="34.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="3"/>
-    <col min="6" max="6" width="67.140625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="14" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="3"/>
+    <col min="5" max="5" width="10.5703125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="3"/>
+    <col min="7" max="7" width="67.140625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="14" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="3"/>
+    <col min="10" max="10" width="67.140625" style="3" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" s="6" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:10" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B1" s="5" t="s">
         <v>40</v>
       </c>
@@ -1813,26 +1867,52 @@
       <c r="D1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="E1" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="str">
-        <f>IF(EXACT(B2, ""), "", CONCATENATE("PERFORM ""SchData-OLTP-Master"".""Func_TblBank_SET""(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, '", B2, "', ", IF(EXACT(C2, ""), "null", CONCATENATE("'", C2, "'")), ", '", D2, "');"))</f>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Mandiri', null, 'BMRIIDJA');</v>
-      </c>
-      <c r="G2" s="2">
+      <c r="E2" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G2" s="3" t="str">
+        <f>IF(EXACT(B2, ""), "", CONCATENATE("PERFORM ""SchData-OLTP-Master"".""Func_TblBank_SET""(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, ", IF(EXACT($B2, ""), "null", CONCATENATE("'", $B2, "'")), ", ", IF(EXACT($C2, ""), "null", CONCATENATE("'", $C2, "'")), ", ", IF(EXACT($D2, ""), "null", CONCATENATE("'", $D2, "'")), ", ", IF(EXACT($E2, ""), "null", CONCATENATE("'", $E2, "'")), ");"))</f>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Mandiri', null, 'BMRIIDJA', 'MRI');</v>
+      </c>
+      <c r="H2" s="2">
         <v>166000000000001</v>
       </c>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="I2" s="34"/>
+      <c r="J2" s="3" t="str">
+        <f>CONCATENATE(
+"varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT (",
+"'recordID', NULL::bigint,", "'entities', ", "JSON_BUILD_OBJECT (",
+"'sysLoginSession_RefID', varSystemLoginSession::bigint,",
+"'sysDataAnnotation', NULL::varchar,",
+"'sysDataSetDateTimeTZ', NULL::timestamptz,",
+"'sysDataValidityStartDateTimeTZ', NULL::timestamptz,",
+"'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,",
+"'sysPartitionRemovableRecordKey_RefID', NULL::bigint,",
+"'sysBranch_RefID', varInstitutionBranchID::bigint,",
+"'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,",
+"'sysDataAnnotation', ", IF(EXACT($B2, ""), "null", CONCATENATE("'", SUBSTITUTE($B2, "'", "\'"), "'")), "::varchar,",
+"'acronym', ", IF(EXACT($C2, ""), "null", CONCATENATE("'", SUBSTITUTE($C2, "'", "\'"), "'")), "::varchar,",
+"'SWIFTCode', ", IF(EXACT($D2, ""), "null", CONCATENATE("'", SUBSTITUTE($D2, "'", "\'"), "'")), "::varchar,",
+"'bankCode', ", IF(EXACT($E2, ""), "null", CONCATENATE("'", SUBSTITUTE($E2, "'", "\'"), "'")), "::varchar",
+")))::varchar;")</f>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Mandiri'::varchar,'acronym', null::varchar,'SWIFTCode', 'BMRIIDJA'::varchar,'bankCode', 'MRI'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1842,15 +1922,38 @@
       <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="3" t="str">
-        <f t="shared" ref="F3:F18" si="0">IF(EXACT(B3, ""), "", CONCATENATE("PERFORM ""SchData-OLTP-Master"".""Func_TblBank_SET""(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, '", B3, "', ", IF(EXACT(C3, ""), "null", CONCATENATE("'", C3, "'")), ", '", D3, "');"))</f>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Rakyat Indonesia', 'BRI', 'BRINIDJA');</v>
-      </c>
-      <c r="G3" s="2">
+      <c r="E3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="3" t="str">
+        <f t="shared" ref="G3:G23" si="0">IF(EXACT(B3, ""), "", CONCATENATE("PERFORM ""SchData-OLTP-Master"".""Func_TblBank_SET""(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, ", IF(EXACT($B3, ""), "null", CONCATENATE("'", $B3, "'")), ", ", IF(EXACT($C3, ""), "null", CONCATENATE("'", $C3, "'")), ", ", IF(EXACT($D3, ""), "null", CONCATENATE("'", $D3, "'")), ", ", IF(EXACT($E3, ""), "null", CONCATENATE("'", $E3, "'")), ");"))</f>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Rakyat Indonesia', 'BRI', 'BRINIDJA', 'BRI');</v>
+      </c>
+      <c r="H3" s="2">
         <v>166000000000002</v>
       </c>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="I3" s="34"/>
+      <c r="J3" s="3" t="str">
+        <f>CONCATENATE(
+"varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT (",
+"'recordID', NULL::bigint,", "'entities', ", "JSON_BUILD_OBJECT (",
+"'sysLoginSession_RefID', varSystemLoginSession::bigint,",
+"'sysDataAnnotation', NULL::varchar,",
+"'sysDataSetDateTimeTZ', NULL::timestamptz,",
+"'sysDataValidityStartDateTimeTZ', NULL::timestamptz,",
+"'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,",
+"'sysPartitionRemovableRecordKey_RefID', NULL::bigint,",
+"'sysBranch_RefID', varInstitutionBranchID::bigint,",
+"'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,",
+"'sysDataAnnotation', ", IF(EXACT($B3, ""), "null", CONCATENATE("'", SUBSTITUTE($B3, "'", "\'"), "'")), "::varchar,",
+"'acronym', ", IF(EXACT($C3, ""), "null", CONCATENATE("'", SUBSTITUTE($C3, "'", "\'"), "'")), "::varchar,",
+"'SWIFTCode', ", IF(EXACT($D3, ""), "null", CONCATENATE("'", SUBSTITUTE($D3, "'", "\'"), "'")), "::varchar,",
+"'bankCode', ", IF(EXACT($E3, ""), "null", CONCATENATE("'", SUBSTITUTE($E3, "'", "\'"), "'")), "::varchar",
+")))::varchar;")</f>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Rakyat Indonesia'::varchar,'acronym', 'BRI'::varchar,'SWIFTCode', 'BRINIDJA'::varchar,'bankCode', 'BRI'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
@@ -1860,15 +1963,37 @@
       <c r="D4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Negara Indonesia', 'BNI', 'BNINIDJA');</v>
-      </c>
-      <c r="G4" s="2">
+      <c r="E4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Negara Indonesia', 'BNI', 'BNINIDJA', 'BNI');</v>
+      </c>
+      <c r="H4" s="2">
         <v>166000000000003</v>
       </c>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J4" s="3" t="str">
+        <f t="shared" ref="J4:J23" si="1">CONCATENATE(
+"varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT (",
+"'recordID', NULL::bigint,", "'entities', ", "JSON_BUILD_OBJECT (",
+"'sysLoginSession_RefID', varSystemLoginSession::bigint,",
+"'sysDataAnnotation', NULL::varchar,",
+"'sysDataSetDateTimeTZ', NULL::timestamptz,",
+"'sysDataValidityStartDateTimeTZ', NULL::timestamptz,",
+"'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,",
+"'sysPartitionRemovableRecordKey_RefID', NULL::bigint,",
+"'sysBranch_RefID', varInstitutionBranchID::bigint,",
+"'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,",
+"'sysDataAnnotation', ", IF(EXACT($B4, ""), "null", CONCATENATE("'", SUBSTITUTE($B4, "'", "\'"), "'")), "::varchar,",
+"'acronym', ", IF(EXACT($C4, ""), "null", CONCATENATE("'", SUBSTITUTE($C4, "'", "\'"), "'")), "::varchar,",
+"'SWIFTCode', ", IF(EXACT($D4, ""), "null", CONCATENATE("'", SUBSTITUTE($D4, "'", "\'"), "'")), "::varchar,",
+"'bankCode', ", IF(EXACT($E4, ""), "null", CONCATENATE("'", SUBSTITUTE($E4, "'", "\'"), "'")), "::varchar",
+")))::varchar;")</f>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Negara Indonesia'::varchar,'acronym', 'BNI'::varchar,'SWIFTCode', 'BNINIDJA'::varchar,'bankCode', 'BNI'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
@@ -1878,15 +2003,22 @@
       <c r="D5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Tabungan Negara', 'BTN', 'BTANIDJA');</v>
-      </c>
-      <c r="G5" s="2">
+      <c r="E5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Tabungan Negara', 'BTN', 'BTANIDJA', 'BTN');</v>
+      </c>
+      <c r="H5" s="2">
         <v>166000000000004</v>
       </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J5" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Tabungan Negara'::varchar,'acronym', 'BTN'::varchar,'SWIFTCode', 'BTANIDJA'::varchar,'bankCode', 'BTN'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
@@ -1896,75 +2028,110 @@
       <c r="D6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Central Asia', 'BCA', 'CENAIDJA');</v>
-      </c>
-      <c r="G6" s="2">
+      <c r="E6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Central Asia', 'BCA', 'CENAIDJA', 'BCA');</v>
+      </c>
+      <c r="H6" s="2">
         <v>166000000000005</v>
       </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J6" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Central Asia'::varchar,'acronym', 'BCA'::varchar,'SWIFTCode', 'CENAIDJA'::varchar,'bankCode', 'BCA'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B7" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Mega', null, 'MEGAIDJA');</v>
-      </c>
-      <c r="G7" s="2">
+      <c r="E7" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Mega', null, 'MEGAIDJA', 'MEG');</v>
+      </c>
+      <c r="H7" s="2">
         <v>166000000000006</v>
       </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J7" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Mega'::varchar,'acronym', null::varchar,'SWIFTCode', 'MEGAIDJA'::varchar,'bankCode', 'MEG'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Permata', null, 'BBBAIDJA');</v>
-      </c>
-      <c r="G8" s="2">
+      <c r="E8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G8" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Permata', null, 'BBBAIDJA', 'PER');</v>
+      </c>
+      <c r="H8" s="2">
         <v>166000000000007</v>
       </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Permata'::varchar,'acronym', null::varchar,'SWIFTCode', 'BBBAIDJA'::varchar,'bankCode', 'PER'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B9" s="3" t="s">
         <v>20</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Danamon', null, 'BDINIDJA');</v>
-      </c>
-      <c r="G9" s="2">
+      <c r="E9" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="G9" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Danamon', null, 'BDINIDJA', 'DAN');</v>
+      </c>
+      <c r="H9" s="2">
         <v>166000000000008</v>
       </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Danamon'::varchar,'acronym', null::varchar,'SWIFTCode', 'BDINIDJA'::varchar,'bankCode', 'DAN'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
         <v>22</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank KB Bukopin', null, 'BBUKIDJA');</v>
-      </c>
-      <c r="G10" s="2">
+      <c r="E10" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank KB Bukopin', null, 'BBUKIDJA', 'BUK');</v>
+      </c>
+      <c r="H10" s="2">
         <v>166000000000009</v>
       </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank KB Bukopin'::varchar,'acronym', null::varchar,'SWIFTCode', 'BBUKIDJA'::varchar,'bankCode', 'BUK'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
@@ -1974,15 +2141,22 @@
       <c r="D11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Syariah Indonesia', 'BSI', 'BSMDIDJA');</v>
-      </c>
-      <c r="G11" s="2">
+      <c r="E11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Syariah Indonesia', 'BSI', 'BSMDIDJA', 'BSI');</v>
+      </c>
+      <c r="H11" s="2">
         <v>166000000000010</v>
       </c>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Syariah Indonesia'::varchar,'acronym', 'BSI'::varchar,'SWIFTCode', 'BSMDIDJA'::varchar,'bankCode', 'BSI'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
         <v>27</v>
       </c>
@@ -1992,15 +2166,22 @@
       <c r="D12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank OCBC Nilai Inti Sari Penyimpanan', 'OCBC NISP', 'NISPIDJA');</v>
-      </c>
-      <c r="G12" s="2">
+      <c r="E12" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank OCBC Nilai Inti Sari Penyimpanan', 'OCBC NISP', 'NISPIDJA', 'OCB');</v>
+      </c>
+      <c r="H12" s="2">
         <v>166000000000011</v>
       </c>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank OCBC Nilai Inti Sari Penyimpanan'::varchar,'acronym', 'OCBC NISP'::varchar,'SWIFTCode', 'NISPIDJA'::varchar,'bankCode', 'OCB'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
         <v>30</v>
       </c>
@@ -2010,45 +2191,66 @@
       <c r="D13" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Tabungan Pensiunan Nasional', 'BTPN', 'SUNIIDJA');</v>
-      </c>
-      <c r="G13" s="2">
+      <c r="E13" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="G13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Tabungan Pensiunan Nasional', 'BTPN', 'SUNIIDJA', 'TPN');</v>
+      </c>
+      <c r="H13" s="2">
         <v>166000000000012</v>
       </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Tabungan Pensiunan Nasional'::varchar,'acronym', 'BTPN'::varchar,'SWIFTCode', 'SUNIIDJA'::varchar,'bankCode', 'TPN'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F14" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pan Indonesia', null, 'PINBIDJA');</v>
-      </c>
-      <c r="G14" s="2">
+      <c r="E14" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G14" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pan Indonesia', null, 'PINBIDJA', 'PAN');</v>
+      </c>
+      <c r="H14" s="2">
         <v>166000000000013</v>
       </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Pan Indonesia'::varchar,'acronym', null::varchar,'SWIFTCode', 'PINBIDJA'::varchar,'bankCode', 'PAN'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
         <v>35</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Maybank Indonesia', null, 'IBBKIDJA');</v>
-      </c>
-      <c r="G15" s="2">
+      <c r="E15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G15" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Maybank Indonesia', null, 'IBBKIDJA', 'MAY');</v>
+      </c>
+      <c r="H15" s="2">
         <v>166000000000014</v>
       </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Maybank Indonesia'::varchar,'acronym', null::varchar,'SWIFTCode', 'IBBKIDJA'::varchar,'bankCode', 'MAY'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B16" s="3" t="s">
         <v>81</v>
       </c>
@@ -2058,66 +2260,94 @@
       <c r="D16" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F16" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Commonwealth', 'Commonwealth', 'BICNIDJA');</v>
-      </c>
-      <c r="G16" s="2">
+      <c r="E16" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="G16" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Commonwealth', 'Commonwealth', 'BICNIDJA', 'CMW');</v>
+      </c>
+      <c r="H16" s="2">
         <v>166000000000015</v>
       </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J16" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Commonwealth'::varchar,'acronym', 'Commonwealth'::varchar,'SWIFTCode', 'BICNIDJA'::varchar,'bankCode', 'CMW'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B17" s="3" t="s">
         <v>84</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="F17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Standard Chartered', null, 'SCBLIDJX');</v>
-      </c>
-      <c r="G17" s="2">
+      <c r="E17" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Standard Chartered', null, 'SCBLIDJX', 'SCD');</v>
+      </c>
+      <c r="H17" s="2">
         <v>166000000000016</v>
       </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J17" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Standard Chartered'::varchar,'acronym', null::varchar,'SWIFTCode', 'SCBLIDJX'::varchar,'bankCode', 'SCD'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B18" s="3" t="s">
         <v>37</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank CIMB Niaga', 'CIMB Niaga', 'BNIAIDJA');</v>
-      </c>
-      <c r="G18" s="2">
+      <c r="E18" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank CIMB Niaga', 'CIMB Niaga', 'BNIAIDJA', 'CIM');</v>
+      </c>
+      <c r="H18" s="2">
         <v>166000000000017</v>
       </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J18" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank CIMB Niaga'::varchar,'acronym', 'CIMB Niaga'::varchar,'SWIFTCode', 'BNIAIDJA'::varchar,'bankCode', 'CIM'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B19" s="3" t="s">
         <v>73</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F19" s="3" t="str">
-        <f t="shared" ref="F19:F21" si="1">IF(EXACT(B19, ""), "", CONCATENATE("PERFORM ""SchData-OLTP-Master"".""Func_TblBank_SET""(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, '", B19, "', ", IF(EXACT(C19, ""), "null", CONCATENATE("'", C19, "'")), ", '", D19, "');"))</f>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Rakyat Indonesia Syariah', 'BRI Syariah', 'BRISIDJA');</v>
-      </c>
-      <c r="G19" s="2">
+      <c r="E19" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="G19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Rakyat Indonesia Syariah', 'BRI Syariah', 'BRISIDJA', 'RIS');</v>
+      </c>
+      <c r="H19" s="2">
         <v>166000000000018</v>
       </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J19" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Rakyat Indonesia Syariah'::varchar,'acronym', 'BRI Syariah'::varchar,'SWIFTCode', 'BRISIDJA'::varchar,'bankCode', 'RIS'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B20" s="3" t="s">
         <v>72</v>
       </c>
@@ -2127,15 +2357,22 @@
       <c r="D20" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="F20" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pembangunan Daerah Bengkulu', 'BPD Bengkulu', 'PDBKIDJ1');</v>
-      </c>
-      <c r="G20" s="2">
+      <c r="E20" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pembangunan Daerah Bengkulu', 'BPD Bengkulu', 'PDBKIDJ1', 'PDB');</v>
+      </c>
+      <c r="H20" s="2">
         <v>166000000000019</v>
       </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J20" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Pembangunan Daerah Bengkulu'::varchar,'acronym', 'BPD Bengkulu'::varchar,'SWIFTCode', 'PDBKIDJ1'::varchar,'bankCode', 'PDB'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B21" s="3" t="s">
         <v>79</v>
       </c>
@@ -2145,15 +2382,22 @@
       <c r="D21" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F21" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pembangunan Daerah Jawa Barat Banten', 'BJB', 'PDJBIDJA');</v>
-      </c>
-      <c r="G21" s="2">
+      <c r="E21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pembangunan Daerah Jawa Barat Banten', 'BJB', 'PDJBIDJA', 'BJB');</v>
+      </c>
+      <c r="H21" s="2">
         <v>166000000000020</v>
       </c>
-    </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J21" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Pembangunan Daerah Jawa Barat Banten'::varchar,'acronym', 'BJB'::varchar,'SWIFTCode', 'PDJBIDJA'::varchar,'bankCode', 'BJB'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B22" s="3" t="s">
         <v>74</v>
       </c>
@@ -2163,15 +2407,22 @@
       <c r="D22" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F22" s="3" t="str">
-        <f t="shared" ref="F22:F23" si="2">IF(EXACT(B22, ""), "", CONCATENATE("PERFORM ""SchData-OLTP-Master"".""Func_TblBank_SET""(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, '", B22, "', ", IF(EXACT(C22, ""), "null", CONCATENATE("'", C22, "'")), ", '", D22, "');"))</f>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pembangunan Daerah Jawa Timur', 'BPD Jatim', 'BJTMIDJA');</v>
-      </c>
-      <c r="G22" s="2">
+      <c r="E22" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pembangunan Daerah Jawa Timur', 'BPD Jatim', 'BJTMIDJA', 'PDJ');</v>
+      </c>
+      <c r="H22" s="2">
         <v>166000000000021</v>
       </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="J22" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Pembangunan Daerah Jawa Timur'::varchar,'acronym', 'BPD Jatim'::varchar,'SWIFTCode', 'BJTMIDJA'::varchar,'bankCode', 'PDJ'::varchar)))::varchar;</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B23" s="3" t="s">
         <v>75</v>
       </c>
@@ -2179,18 +2430,26 @@
         <v>78</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="F23" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null, null, null, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pembangunan Daerah Kalimantan Selatan', 'BPD Kalsel', ' PDKSIDJ1');</v>
-      </c>
-      <c r="G23" s="2">
+        <v>94</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="G23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v>PERFORM "SchData-OLTP-Master"."Func_TblBank_SET"(varSystemLoginSession, null::bigint, null::varchar, null::varchar, varInstitutionBranchID, varBaseCurrencyID, 'Bank Pembangunan Daerah Kalimantan Selatan', 'BPD Kalsel', 'PDKSIDJ1', 'PDK');</v>
+      </c>
+      <c r="H23" s="2">
         <v>166000000000022</v>
+      </c>
+      <c r="J23" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>varSQL := varSQL || (CASE WHEN (varSQL = '') THEN '' ELSE ', ' END) || (SELECT JSON_BUILD_OBJECT ('recordID', NULL::bigint,'entities', JSON_BUILD_OBJECT ('sysLoginSession_RefID', varSystemLoginSession::bigint,'sysDataAnnotation', NULL::varchar,'sysDataSetDateTimeTZ', NULL::timestamptz,'sysDataValidityStartDateTimeTZ', NULL::timestamptz,'sysDataValidityFinishDateTimeTZ', NULL::timestamptz,'sysPartitionRemovableRecordKey_RefID', NULL::bigint,'sysBranch_RefID', varInstitutionBranchID::bigint,'sysBaseCurrency_RefID',varBaseCurrencyID::bigint,'sysDataAnnotation', 'Bank Pembangunan Daerah Kalimantan Selatan'::varchar,'acronym', 'BPD Kalsel'::varchar,'SWIFTCode', 'PDKSIDJ1'::varchar,'bankCode', 'PDK'::varchar)))::varchar;</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>